<commit_message>
Integra 3 funcionalidades al proyecto
- Agrega modo "pantalla en casa" (tablet + Fully Kiosk Browser),
  integración con pulsera inteligente (Health Connect) y detección
  de ruido fuerte (micrófono del dispositivo) como respuesta al
  pedido del docente de diferenciar el proyecto
- 1.5: nuevos objetivos específicos, sección de diferenciadores,
  nota de factibilidad, y actividades agregadas a Plan de Trabajo
  y Carta Gantt (semanas 13-15)
- PPT: nueva slide de diferenciadores; guion actualizado
- Se evitó fabricar hardware propio (sensor de sonido dedicado):
  se prioriza tecnología de bajo costo ya existente en el mercado
- Product Backlog: extiende la historia "Interfaz simplificada" para
  incluir el modo pantalla en casa; agrega 2 épicas nuevas (pulsera
  inteligente, detección de ruido)
- Cronograma Semestral: menciona las 3 funciones en semanas 13-15,
  coherente con la Carta Gantt del 1.5
</commit_message>
<xml_diff>
--- a/Fase 1/Evidencias Grupales/Cronograma_Actividades_Equipo_PerfilMedico.xlsx
+++ b/Fase 1/Evidencias Grupales/Cronograma_Actividades_Equipo_PerfilMedico.xlsx
@@ -1102,7 +1102,7 @@
       </c>
       <c r="F17" s="12" t="inlineStr">
         <is>
-          <t>Historial de cumplimiento y gráficos de indicadores (BD + Backend). Botón de asistencia (App)</t>
+          <t>Historial de cumplimiento y gráficos de indicadores (BD + Backend). Botón de asistencia (App). Modo "pantalla en casa" sobre tablet fija (App)</t>
         </is>
       </c>
       <c r="G17" s="12" t="inlineStr">
@@ -1138,7 +1138,7 @@
       </c>
       <c r="F18" s="12" t="inlineStr">
         <is>
-          <t>Módulo de IA — orientación general (integración API LLM) y detección simple de patrones (BD + IA)</t>
+          <t>Módulo de IA — orientación general (integración API LLM) y detección simple de patrones (BD + IA). Integración con pulsera inteligente vía Health Connect (BD + Backend)</t>
         </is>
       </c>
       <c r="G18" s="12" t="inlineStr">
@@ -1174,7 +1174,7 @@
       </c>
       <c r="F19" s="12" t="inlineStr">
         <is>
-          <t>Pruebas integrales, ajustes finales, documentación (manual técnico, Docker) y presentación del Informe Final</t>
+          <t>Detección de sonidos fuertes vía micrófono del dispositivo (App). Pruebas integrales, ajustes finales, documentación (manual técnico, Docker) y presentación del Informe Final</t>
         </is>
       </c>
       <c r="G19" s="12" t="inlineStr">
@@ -1312,7 +1312,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1331,7 +1331,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -1730,7 +1729,7 @@
       </c>
       <c r="C14" s="20" t="inlineStr">
         <is>
-          <t>Como perfil dependiente (ej. adulto mayor) quiero una interfaz simplificada con botones grandes y confirmación en un toque</t>
+          <t>Como perfil dependiente (ej. adulto mayor) quiero una interfaz simplificada con botones grandes y confirmación en un toque, disponible también en modo "pantalla en casa" sobre una tablet fija (vía Fully Kiosk Browser) para quienes no manejan un smartphone</t>
         </is>
       </c>
       <c r="D14" s="19" t="inlineStr">
@@ -1926,6 +1925,76 @@
       <c r="G19" s="19" t="inlineStr">
         <is>
           <t>Alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>17</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Pulsera inteligente</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Como titular o cuidador quiero ver signos vitales (frecuencia cardíaca) de un perfil desde una pulsera inteligente conectada, sin instrumentación adicional</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Perfil (titular/dependiente)</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Sergio (BD) / Benjamín (Backend)</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>18</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Detección de ruido</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Como cuidador quiero recibir una alerta si el dispositivo del perfil dependiente detecta un sonido fuerte en el hogar (posible caída)</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Perfil dependiente</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Matías (App) / Benjamín (Backend)</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Sprint 6</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Media</t>
         </is>
       </c>
     </row>
@@ -1960,7 +2029,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -2049,7 +2117,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>

</xml_diff>